<commit_message>
Ensure 8-column appointment bookings format (Date & Time, Customer Name, Customer Email, Customer Phone, Staff Name, Service, Duration (mins.), Status) for import, export, and sample template
</commit_message>
<xml_diff>
--- a/SSS_Toledo_Sample_Appointment_Bookings.xlsx
+++ b/SSS_Toledo_Sample_Appointment_Bookings.xlsx
@@ -37,7 +37,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>2026-08-27 08:30 AM</t>
+    <t>2026-08-29 08:30 AM</t>
   </si>
   <si>
     <t>Juan dela Cruz</t>
@@ -58,7 +58,7 @@
     <t>Confirmed</t>
   </si>
   <si>
-    <t>2026-08-27 09:00 AM</t>
+    <t>2026-08-29 09:00 AM</t>
   </si>
   <si>
     <t>Maria Clara Santos</t>
@@ -76,7 +76,7 @@
     <t>Maternity Benefit Claim</t>
   </si>
   <si>
-    <t>2026-08-27 09:30 AM</t>
+    <t>2026-08-29 09:30 AM</t>
   </si>
   <si>
     <t>Jose P. Rizal</t>
@@ -94,7 +94,7 @@
     <t>Retirement Benefit Claim</t>
   </si>
   <si>
-    <t>2026-08-27 10:00 AM</t>
+    <t>2026-08-29 10:00 AM</t>
   </si>
   <si>
     <t>Andres Bonifacio</t>
@@ -112,7 +112,7 @@
     <t>Sickness Benefit Claim</t>
   </si>
   <si>
-    <t>2026-08-27 10:30 AM</t>
+    <t>2026-08-29 10:30 AM</t>
   </si>
   <si>
     <t>Teresa Magbanua</t>
@@ -130,7 +130,7 @@
     <t>Senior Citizen / Pensioner Assistance</t>
   </si>
   <si>
-    <t>2026-08-27 11:00 AM</t>
+    <t>2026-08-29 11:00 AM</t>
   </si>
   <si>
     <t>Emilio Aguinaldo</t>
@@ -145,7 +145,7 @@
     <t>Death / Funeral Claim</t>
   </si>
   <si>
-    <t>2026-08-27 01:30 PM</t>
+    <t>2026-08-29 01:30 PM</t>
   </si>
   <si>
     <t>Melchora Aquino</t>
@@ -160,7 +160,7 @@
     <t>Senior Citizen / Pension Inquiry</t>
   </si>
   <si>
-    <t>2026-08-27 02:00 PM</t>
+    <t>2026-08-29 02:00 PM</t>
   </si>
   <si>
     <t>Antonio Luna</t>
@@ -175,7 +175,7 @@
     <t>Salary / Calamity Loan Application</t>
   </si>
   <si>
-    <t>2026-08-27 02:30 PM</t>
+    <t>2026-08-29 02:30 PM</t>
   </si>
   <si>
     <t>Gabriela Silang</t>
@@ -187,7 +187,7 @@
     <t>09216667788</t>
   </si>
   <si>
-    <t>2026-08-27 03:00 PM</t>
+    <t>2026-08-29 03:00 PM</t>
   </si>
   <si>
     <t>Apolinario Mabini</t>

</xml_diff>

<commit_message>
Update official staff roster to Christie Sillar, Noeme Mamac, Glory May Tagpuno, Emmie Flores, Mabelle Paz, and Maricar Boniao
</commit_message>
<xml_diff>
--- a/SSS_Toledo_Sample_Appointment_Bookings.xlsx
+++ b/SSS_Toledo_Sample_Appointment_Bookings.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
   <si>
     <t>Date &amp; Time</t>
   </si>
@@ -70,7 +70,7 @@
     <t>09289876543</t>
   </si>
   <si>
-    <t>Marga Ursal</t>
+    <t>Noeme Mamac</t>
   </si>
   <si>
     <t>Maternity Benefit Claim</t>
@@ -88,7 +88,7 @@
     <t>09185551234</t>
   </si>
   <si>
-    <t>Laarnie Alibong</t>
+    <t>Glory May Tagpuno</t>
   </si>
   <si>
     <t>Retirement Benefit Claim</t>
@@ -106,7 +106,7 @@
     <t>09228889900</t>
   </si>
   <si>
-    <t>Sheina Torrecampo</t>
+    <t>Emmie Flores</t>
   </si>
   <si>
     <t>Sickness Benefit Claim</t>
@@ -124,7 +124,7 @@
     <t>09191112233</t>
   </si>
   <si>
-    <t>Sheila Vasquez</t>
+    <t>Mabelle Paz</t>
   </si>
   <si>
     <t>Senior Citizen / Pensioner Assistance</t>
@@ -142,6 +142,9 @@
     <t>09173334455</t>
   </si>
   <si>
+    <t>Maricar Boniao</t>
+  </si>
+  <si>
     <t>Death / Funeral Claim</t>
   </si>
   <si>
@@ -200,6 +203,36 @@
   </si>
   <si>
     <t>Disability Benefit Claim</t>
+  </si>
+  <si>
+    <t>2026-08-29 03:30 PM</t>
+  </si>
+  <si>
+    <t>Francisco Baltazar</t>
+  </si>
+  <si>
+    <t>balagtas.francisco@gmail.com</t>
+  </si>
+  <si>
+    <t>09192223344</t>
+  </si>
+  <si>
+    <t>Contribution Verification / Inquiries</t>
+  </si>
+  <si>
+    <t>2026-08-29 04:00 PM</t>
+  </si>
+  <si>
+    <t>Diego Silang</t>
+  </si>
+  <si>
+    <t>diego.silang@history.ph</t>
+  </si>
+  <si>
+    <t>09178881234</t>
+  </si>
+  <si>
+    <t>Payment &amp; PRN Verification</t>
   </si>
 </sst>
 </file>
@@ -659,7 +692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -842,10 +875,10 @@
         <v>42</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G7" s="5">
         <v>25</v>
@@ -856,22 +889,22 @@
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" s="2">
         <v>15</v>
@@ -882,22 +915,22 @@
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>25</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G9" s="5">
         <v>15</v>
@@ -908,16 +941,16 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>31</v>
@@ -934,27 +967,79 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>37</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G11" s="5">
         <v>20</v>
       </c>
       <c r="H11" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="2">
+        <v>15</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="5">
+        <v>15</v>
+      </c>
+      <c r="H13" s="7" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>